<commit_message>
Initial Commit - 2
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -25,12 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2744" uniqueCount="749">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2749" uniqueCount="752">
   <si>
     <t>PII Service — API test cases by endpoint</t>
   </si>
   <si>
-    <t>Generated from the code with "npm run docs:testcases" on 2026-09-26. Last result from: local (no service) 2026-09-26 14:15 UTC. Click an endpoint to open its tab.</t>
+    <t>Generated from the code with "npm run docs:testcases" on 2026-09-26. Last result from: local (no service) 2026-09-26 14:37 UTC. Click an endpoint to open its tab.</t>
   </si>
   <si>
     <t>#</t>
@@ -150,7 +150,7 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Framework self-tests (no service needed): 81 — see the "Self-tests" tab.</t>
+    <t>Framework self-tests (no service needed): 82 — see the "Self-tests" tab.</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -381,7 +381,7 @@
     <t>Q-21</t>
   </si>
   <si>
-    <t>tests/security/authentication.spec.ts:257</t>
+    <t>tests/security/authentication.spec.ts:258</t>
   </si>
   <si>
     <t>PII-AZ-001</t>
@@ -441,7 +441,7 @@
     <t>Emails are saved without surrounding spaces and in lower case</t>
   </si>
   <si>
-    <t>tests/pii/normalization.spec.ts:37</t>
+    <t>tests/pii/normalization.spec.ts:36</t>
   </si>
   <si>
     <t>PII-NRM-002</t>
@@ -450,7 +450,7 @@
     <t>Phones are saved as digits only (spaces, dashes, brackets and + removed)</t>
   </si>
   <si>
-    <t>tests/pii/normalization.spec.ts:52</t>
+    <t>tests/pii/normalization.spec.ts:51</t>
   </si>
   <si>
     <t>PII-NRM-003</t>
@@ -459,7 +459,7 @@
     <t>Names are trimmed and repeated spaces collapsed; upper/lower case is kept</t>
   </si>
   <si>
-    <t>tests/pii/normalization.spec.ts:68</t>
+    <t>tests/pii/normalization.spec.ts:67</t>
   </si>
   <si>
     <t>PII-NRM-004</t>
@@ -468,7 +468,7 @@
     <t>Phones with exactly 8 and exactly 15 digits (the allowed limits) are accepted</t>
   </si>
   <si>
-    <t>tests/pii/normalization.spec.ts:84</t>
+    <t>tests/pii/normalization.spec.ts:83</t>
   </si>
   <si>
     <t>PII-NRM-005</t>
@@ -477,7 +477,7 @@
     <t>Values that are already clean are saved unchanged</t>
   </si>
   <si>
-    <t>tests/pii/normalization.spec.ts:114</t>
+    <t>tests/pii/normalization.spec.ts:113</t>
   </si>
   <si>
     <t>PII-SEC-001</t>
@@ -1722,7 +1722,7 @@
     <t>UT-CLI-002</t>
   </si>
   <si>
-    <t>Every request carries the four documented headers with correct values</t>
+    <t>Every request carries the documented headers (guide + tech doc) with correct values</t>
   </si>
   <si>
     <t>tests/unit/pii-client-wire.spec.ts:61</t>
@@ -1734,7 +1734,7 @@
     <t>Every request gets a new, unique request ID</t>
   </si>
   <si>
-    <t>tests/unit/pii-client-wire.spec.ts:72</t>
+    <t>tests/unit/pii-client-wire.spec.ts:77</t>
   </si>
   <si>
     <t>UT-CLI-004</t>
@@ -1743,7 +1743,7 @@
     <t>The search field name is safely encoded into the URL</t>
   </si>
   <si>
-    <t>tests/unit/pii-client-wire.spec.ts:79</t>
+    <t>tests/unit/pii-client-wire.spec.ts:84</t>
   </si>
   <si>
     <t>UT-CLI-005</t>
@@ -1752,7 +1752,7 @@
     <t>The health check is sent without security headers or a body</t>
   </si>
   <si>
-    <t>tests/unit/pii-client-wire.spec.ts:88</t>
+    <t>tests/unit/pii-client-wire.spec.ts:93</t>
   </si>
   <si>
     <t>UT-CLI-006</t>
@@ -1761,7 +1761,7 @@
     <t>Tests can remove headers, and no Content-Type is added behind their back</t>
   </si>
   <si>
-    <t>tests/unit/pii-client-wire.spec.ts:97</t>
+    <t>tests/unit/pii-client-wire.spec.ts:103</t>
   </si>
   <si>
     <t>UT-CLI-007</t>
@@ -1770,7 +1770,7 @@
     <t>Tests can deliberately send a body that differs from what was signed</t>
   </si>
   <si>
-    <t>tests/unit/pii-client-wire.spec.ts:108</t>
+    <t>tests/unit/pii-client-wire.spec.ts:115</t>
   </si>
   <si>
     <t>UT-CLI-008</t>
@@ -1779,7 +1779,7 @@
     <t>Tests can sign with another key or the wrong method while keeping the caller ID</t>
   </si>
   <si>
-    <t>tests/unit/pii-client-wire.spec.ts:120</t>
+    <t>tests/unit/pii-client-wire.spec.ts:127</t>
   </si>
   <si>
     <t>UT-CLI-009</t>
@@ -1788,7 +1788,7 @@
     <t>Read-only calls retry on 503 with a new request ID, a limited number of times</t>
   </si>
   <si>
-    <t>tests/unit/pii-client-wire.spec.ts:134</t>
+    <t>tests/unit/pii-client-wire.spec.ts:141</t>
   </si>
   <si>
     <t>UT-CLI-010</t>
@@ -1797,7 +1797,7 @@
     <t>Saves are never retried, and 401/403 responses are never retried</t>
   </si>
   <si>
-    <t>tests/unit/pii-client-wire.spec.ts:151</t>
+    <t>tests/unit/pii-client-wire.spec.ts:158</t>
   </si>
   <si>
     <t>UT-CLI-011</t>
@@ -1806,7 +1806,7 @@
     <t>Non-JSON and empty responses are handled, and response bodies are never printed</t>
   </si>
   <si>
-    <t>tests/unit/pii-client-wire.spec.ts:172</t>
+    <t>tests/unit/pii-client-wire.spec.ts:179</t>
   </si>
   <si>
     <t>UT-CLI-012</t>
@@ -1815,7 +1815,7 @@
     <t>Logs contain request details but no personal data, signatures or bodies</t>
   </si>
   <si>
-    <t>tests/unit/pii-client-wire.spec.ts:194</t>
+    <t>tests/unit/pii-client-wire.spec.ts:201</t>
   </si>
   <si>
     <t>UT-CLI-013</t>
@@ -1824,7 +1824,7 @@
     <t>Calling a signed endpoint with no caller set up fails early with a clear message</t>
   </si>
   <si>
-    <t>tests/unit/pii-client-wire.spec.ts:205</t>
+    <t>tests/unit/pii-client-wire.spec.ts:212</t>
   </si>
   <si>
     <t>UT-CLI-014</t>
@@ -1833,7 +1833,7 @@
     <t>Network errors are reported without the request body or headers</t>
   </si>
   <si>
-    <t>tests/unit/pii-client-wire.spec.ts:216</t>
+    <t>tests/unit/pii-client-wire.spec.ts:223</t>
   </si>
   <si>
     <t>UT-CLI-015</t>
@@ -1842,7 +1842,7 @@
     <t>Every logged call is labelled as test, setup or verification</t>
   </si>
   <si>
-    <t>tests/unit/pii-client-wire.spec.ts:225</t>
+    <t>tests/unit/pii-client-wire.spec.ts:232</t>
   </si>
   <si>
     <t>Clean-up</t>
@@ -2122,6 +2122,15 @@
   </si>
   <si>
     <t>tests/unit/redaction-logger.spec.ts:91</t>
+  </si>
+  <si>
+    <t>UT-RED-008</t>
+  </si>
+  <si>
+    <t>The body-hash header (an unkeyed hash of PII) is never logged, by key or as free text</t>
+  </si>
+  <si>
+    <t>tests/unit/redaction-logger.spec.ts:115</t>
   </si>
   <si>
     <t>Retries</t>
@@ -4293,7 +4302,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E83"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -4704,8 +4713,8 @@
       <c r="C24" s="13" t="s">
         <v>565</v>
       </c>
-      <c r="D24" s="22" t="s">
-        <v>9</v>
+      <c r="D24" s="14" t="s">
+        <v>11</v>
       </c>
       <c r="E24" s="15" t="s">
         <v>566</v>
@@ -5427,24 +5436,24 @@
     </row>
     <row r="67" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="17" t="s">
+        <v>674</v>
+      </c>
+      <c r="B67" s="16" t="s">
         <v>699</v>
       </c>
-      <c r="B67" s="16" t="s">
+      <c r="C67" s="17" t="s">
         <v>700</v>
       </c>
-      <c r="C67" s="17" t="s">
+      <c r="D67" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E67" s="19" t="s">
         <v>701</v>
-      </c>
-      <c r="D67" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="E67" s="19" t="s">
-        <v>702</v>
       </c>
     </row>
     <row r="68" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="13" t="s">
-        <v>699</v>
+        <v>702</v>
       </c>
       <c r="B68" s="12" t="s">
         <v>703</v>
@@ -5461,24 +5470,24 @@
     </row>
     <row r="69" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="17" t="s">
+        <v>702</v>
+      </c>
+      <c r="B69" s="16" t="s">
         <v>706</v>
       </c>
-      <c r="B69" s="16" t="s">
+      <c r="C69" s="17" t="s">
         <v>707</v>
-      </c>
-      <c r="C69" s="17" t="s">
-        <v>708</v>
       </c>
       <c r="D69" s="23" t="s">
         <v>9</v>
       </c>
       <c r="E69" s="19" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="70" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="13" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B70" s="12" t="s">
         <v>710</v>
@@ -5495,7 +5504,7 @@
     </row>
     <row r="71" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="17" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B71" s="16" t="s">
         <v>713</v>
@@ -5512,7 +5521,7 @@
     </row>
     <row r="72" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="13" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B72" s="12" t="s">
         <v>716</v>
@@ -5529,7 +5538,7 @@
     </row>
     <row r="73" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="17" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B73" s="16" t="s">
         <v>719</v>
@@ -5546,7 +5555,7 @@
     </row>
     <row r="74" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="13" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B74" s="12" t="s">
         <v>722</v>
@@ -5563,7 +5572,7 @@
     </row>
     <row r="75" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="17" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B75" s="16" t="s">
         <v>725</v>
@@ -5580,7 +5589,7 @@
     </row>
     <row r="76" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="13" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B76" s="12" t="s">
         <v>728</v>
@@ -5597,7 +5606,7 @@
     </row>
     <row r="77" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="17" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B77" s="16" t="s">
         <v>731</v>
@@ -5614,7 +5623,7 @@
     </row>
     <row r="78" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="13" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B78" s="12" t="s">
         <v>734</v>
@@ -5631,7 +5640,7 @@
     </row>
     <row r="79" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="17" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B79" s="16" t="s">
         <v>737</v>
@@ -5648,7 +5657,7 @@
     </row>
     <row r="80" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="13" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B80" s="12" t="s">
         <v>740</v>
@@ -5665,7 +5674,7 @@
     </row>
     <row r="81" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="17" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B81" s="16" t="s">
         <v>743</v>
@@ -5682,7 +5691,7 @@
     </row>
     <row r="82" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="13" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B82" s="12" t="s">
         <v>746</v>
@@ -5695,6 +5704,23 @@
       </c>
       <c r="E82" s="15" t="s">
         <v>748</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="17" t="s">
+        <v>709</v>
+      </c>
+      <c r="B83" s="16" t="s">
+        <v>749</v>
+      </c>
+      <c r="C83" s="17" t="s">
+        <v>750</v>
+      </c>
+      <c r="D83" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="E83" s="19" t="s">
+        <v>751</v>
       </c>
     </row>
   </sheetData>

</xml_diff>